<commit_message>
Updated April 8 hikes
</commit_message>
<xml_diff>
--- a/portfolio/posts/_data/Flynn_Dam_Heights.xlsx
+++ b/portfolio/posts/_data/Flynn_Dam_Heights.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1590" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1597" uniqueCount="142">
   <si>
     <t>DateTime</t>
   </si>
@@ -773,7 +773,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1154"/>
+  <dimension ref="A1:E1159"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -15935,7 +15935,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="1153" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1153" t="s">
         <v>135</v>
       </c>
@@ -15946,7 +15946,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="1154" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1154" t="s">
         <v>135</v>
       </c>
@@ -15958,6 +15958,70 @@
       </c>
       <c r="D1154">
         <v>0.01</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1155" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1155" s="1">
+        <v>46198.430555555555</v>
+      </c>
+      <c r="C1155" s="2">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1156" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1156" s="1">
+        <v>46199.736805555556</v>
+      </c>
+      <c r="C1156" s="2">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1157" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1157" s="1">
+        <v>46200.5</v>
+      </c>
+      <c r="C1157" s="2">
+        <v>1.75</v>
+      </c>
+      <c r="E1157" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1158" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1158" s="1">
+        <v>46201.53402777778</v>
+      </c>
+      <c r="C1158" s="2">
+        <v>1.74</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1159" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1159" s="1">
+        <v>46202.615972222222</v>
+      </c>
+      <c r="C1159" s="2">
+        <v>1.76</v>
+      </c>
+      <c r="D1159">
+        <v>0.12</v>
+      </c>
+      <c r="E1159" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finally finished Hawaii Trails
</commit_message>
<xml_diff>
--- a/portfolio/posts/_data/Flynn_Dam_Heights.xlsx
+++ b/portfolio/posts/_data/Flynn_Dam_Heights.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1597" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="142">
   <si>
     <t>DateTime</t>
   </si>
@@ -773,7 +773,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1159"/>
+  <dimension ref="A1:E1168"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -16024,6 +16024,117 @@
         <v>117</v>
       </c>
     </row>
+    <row r="1160" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1160" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1160" s="1">
+        <v>46203.369444444441</v>
+      </c>
+      <c r="C1160" s="2">
+        <v>1.85</v>
+      </c>
+      <c r="D1160">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1161" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1161" s="1">
+        <v>46204.589583333334</v>
+      </c>
+      <c r="C1161" s="2">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1162" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1162" s="1">
+        <v>46205.429166666669</v>
+      </c>
+      <c r="C1162" s="2">
+        <v>1.83</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1163" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1163" s="1">
+        <v>46206.506944444445</v>
+      </c>
+      <c r="C1163" s="2">
+        <v>1.81</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1164" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1164" s="1">
+        <v>46207.397916666669</v>
+      </c>
+      <c r="C1164" s="2">
+        <v>1.82</v>
+      </c>
+      <c r="D1164">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1165" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1165" s="1">
+        <v>46208.613194444442</v>
+      </c>
+      <c r="C1165" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1166" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1166" s="1">
+        <v>46209.575694444444</v>
+      </c>
+      <c r="C1166" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1167" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1167" s="1">
+        <v>46210.756944444445</v>
+      </c>
+      <c r="C1167" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="D1167">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1168" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1168" s="1">
+        <v>46211.430555555555</v>
+      </c>
+      <c r="C1168" s="2">
+        <v>1.82</v>
+      </c>
+      <c r="D1168">
+        <v>0.32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>